<commit_message>
Fix FRCoreValueSetAllergyCode : restreindre CIM-11 au bloc Chapitre X pertinent
L'inclusion CIM-11 référençait toute la MMS (36480 concepts) via l'URL WHO
brute, au lieu de se limiter au Chapitre X Extensions. Filtre désormais sur
le bloc XM9N55 "Substances, essentiellement non médicinales" (aliments,
agents chimiques/environnementaux/physiques/biologiques), via le miroir
ANS SMT, cohérent avec les ValueSets FRCoreValueSetAllergyIntoleranceManifestation*.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> 7241fa57dc457e0ad4c29ec5a5171d3f55f1b86a
</commit_message>
<xml_diff>
--- a/nr-doc-core-allergy-intolerance/ig/ValueSet-fr-core-vs-allergy-code.xlsx
+++ b/nr-doc-core-allergy-intolerance/ig/ValueSet-fr-core-vs-allergy-code.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="43">
   <si>
     <t>Property</t>
   </si>
@@ -64,7 +64,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-13T15:20:13+00:00</t>
+    <t>2026-10-13T15:41:31+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -129,7 +129,19 @@
     <t>https://smt.esante.gouv.fr/terminologie-cip_ucd</t>
   </si>
   <si>
-    <t>http://id.who.int/icd/release/11/mms</t>
+    <t>Operation</t>
+  </si>
+  <si>
+    <t>concept</t>
+  </si>
+  <si>
+    <t>is-a</t>
+  </si>
+  <si>
+    <t>XM9N55</t>
+  </si>
+  <si>
+    <t>https://smt.esante.gouv.fr/terminologie-cim11-mms</t>
   </si>
   <si>
     <t>ValueSet URL</t>
@@ -490,7 +502,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="30.703125" customWidth="true"/>
@@ -499,12 +511,24 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="1">
-        <v>29</v>
+        <v>0</v>
+      </c>
+      <c r="B1" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="C1" t="s" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>30</v>
+        <v>36</v>
+      </c>
+      <c r="B2" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="C2" t="s" s="2">
+        <v>38</v>
       </c>
     </row>
     <row r="3">
@@ -520,7 +544,7 @@
         <v>32</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -539,12 +563,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="1">
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -584,7 +608,7 @@
         <v>32</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>